<commit_message>
Updated sprint backlog with my assigned tasks
</commit_message>
<xml_diff>
--- a/MealPlanner/sprints/sprint1/Sprint Backlog & Burnup Chart.xlsx
+++ b/MealPlanner/sprints/sprint1/Sprint Backlog & Burnup Chart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29728"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westga365-my.sharepoint.com/personal/jcorley_westga_edu/Documents/Teaching/Software Engineering II/SE2 - Spring 2026/Project/SE2-project-repos-sample/sprints/sprint1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a648f88e637c48b0/Coding Stuff/School/Software Engineering/Semester 2/MealPlanner/MealPlanner/sprints/sprint1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{66AE5F6F-FD3B-4C83-AE1C-1436BAD6C7C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{66AE5F6F-FD3B-4C83-AE1C-1436BAD6C7C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5E09801-2189-4B2F-BD20-ADE8C081F215}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -95,9 +95,6 @@
     <t>Make model class for meal</t>
   </si>
   <si>
-    <t>View planner</t>
-  </si>
-  <si>
     <t>Make view for viewing planner</t>
   </si>
   <si>
@@ -126,13 +123,16 @@
   </si>
   <si>
     <t>Estimate Totals</t>
+  </si>
+  <si>
+    <t>View planner (Kirya)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1423,14 +1423,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G28"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="51.42578125" customWidth="1"/>
     <col min="2" max="2" width="41.7109375" customWidth="1"/>
     <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -1447,7 +1447,7 @@
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="7"/>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
@@ -1464,7 +1464,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -1479,7 +1479,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1494,7 +1494,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -1509,7 +1509,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -1524,7 +1524,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -1539,7 +1539,7 @@
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>12</v>
       </c>
@@ -1554,7 +1554,7 @@
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -1569,7 +1569,7 @@
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -1584,12 +1584,12 @@
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="C11" s="1">
         <v>0.5</v>
@@ -1599,12 +1599,12 @@
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C12" s="1">
         <v>1.5</v>
@@ -1614,12 +1614,12 @@
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C13" s="1">
         <v>1</v>
@@ -1629,12 +1629,12 @@
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="C14" s="1">
         <v>1.5</v>
@@ -1644,12 +1644,12 @@
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="C15" s="1">
         <v>0.5</v>
@@ -1659,12 +1659,12 @@
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C16" s="1">
         <v>1</v>
@@ -1674,12 +1674,12 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C17" s="1">
         <v>1</v>
@@ -1689,7 +1689,7 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -1698,7 +1698,7 @@
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -1707,7 +1707,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -1716,7 +1716,7 @@
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -1725,7 +1725,7 @@
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -1734,7 +1734,7 @@
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1743,7 +1743,7 @@
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -1752,7 +1752,7 @@
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -1761,7 +1761,7 @@
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1770,9 +1770,9 @@
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B27" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C27" s="3">
         <f>SUM(C3:C26)</f>
@@ -1795,7 +1795,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D28">
         <f>$C$27</f>
         <v>14</v>

</xml_diff>

<commit_message>
Reverted the first pull request to remove uneeded files. Revert "Merge pull request #3 from JarethUWG/SetupMavenProject"
This reverts commit 4ec42660898b3326b14470ebb21d17659b32c73d, reversing
changes made to 64bc6bdc1a0f0407d021a4b913bfb45cb65f4c8a.
</commit_message>
<xml_diff>
--- a/MealPlanner/sprints/sprint1/Sprint Backlog & Burnup Chart.xlsx
+++ b/MealPlanner/sprints/sprint1/Sprint Backlog & Burnup Chart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29728"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a648f88e637c48b0/Coding Stuff/School/Software Engineering/Semester 2/MealPlanner/MealPlanner/sprints/sprint1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westga365-my.sharepoint.com/personal/jcorley_westga_edu/Documents/Teaching/Software Engineering II/SE2 - Spring 2026/Project/SE2-project-repos-sample/sprints/sprint1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{66AE5F6F-FD3B-4C83-AE1C-1436BAD6C7C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5E09801-2189-4B2F-BD20-ADE8C081F215}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{66AE5F6F-FD3B-4C83-AE1C-1436BAD6C7C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -95,6 +95,9 @@
     <t>Make model class for meal</t>
   </si>
   <si>
+    <t>View planner</t>
+  </si>
+  <si>
     <t>Make view for viewing planner</t>
   </si>
   <si>
@@ -123,16 +126,13 @@
   </si>
   <si>
     <t>Estimate Totals</t>
-  </si>
-  <si>
-    <t>View planner (Kirya)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1423,14 +1423,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="51.42578125" customWidth="1"/>
     <col min="2" max="2" width="41.7109375" customWidth="1"/>
     <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -1447,7 +1447,7 @@
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="A2" s="7"/>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
@@ -1464,7 +1464,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -1479,7 +1479,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1494,7 +1494,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -1509,7 +1509,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -1524,7 +1524,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -1539,7 +1539,7 @@
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" s="1" t="s">
         <v>12</v>
       </c>
@@ -1554,7 +1554,7 @@
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -1569,7 +1569,7 @@
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -1584,12 +1584,12 @@
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="A11" s="1" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C11" s="1">
         <v>0.5</v>
@@ -1599,12 +1599,12 @@
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="A12" s="1" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C12" s="1">
         <v>1.5</v>
@@ -1614,12 +1614,12 @@
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7">
       <c r="A13" s="1" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C13" s="1">
         <v>1</v>
@@ -1629,12 +1629,12 @@
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7">
       <c r="A14" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C14" s="1">
         <v>1.5</v>
@@ -1644,12 +1644,12 @@
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="A15" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C15" s="1">
         <v>0.5</v>
@@ -1659,12 +1659,12 @@
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="A16" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C16" s="1">
         <v>1</v>
@@ -1674,12 +1674,12 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7">
       <c r="A17" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C17" s="1">
         <v>1</v>
@@ -1689,7 +1689,7 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -1698,7 +1698,7 @@
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -1707,7 +1707,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -1716,7 +1716,7 @@
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -1725,7 +1725,7 @@
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -1734,7 +1734,7 @@
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1743,7 +1743,7 @@
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -1752,7 +1752,7 @@
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -1761,7 +1761,7 @@
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1770,9 +1770,9 @@
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7">
       <c r="B27" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C27" s="3">
         <f>SUM(C3:C26)</f>
@@ -1795,7 +1795,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7">
       <c r="D28">
         <f>$C$27</f>
         <v>14</v>

</xml_diff>

<commit_message>
Added basic planner view window
Updated sprint chart with my assigned tasks
</commit_message>
<xml_diff>
--- a/MealPlanner/sprints/sprint1/Sprint Backlog & Burnup Chart.xlsx
+++ b/MealPlanner/sprints/sprint1/Sprint Backlog & Burnup Chart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29728"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westga365-my.sharepoint.com/personal/jcorley_westga_edu/Documents/Teaching/Software Engineering II/SE2 - Spring 2026/Project/SE2-project-repos-sample/sprints/sprint1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kirya\git\MealPlanner-CS3212-Group4\MealPlanner\sprints\sprint1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{66AE5F6F-FD3B-4C83-AE1C-1436BAD6C7C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6856656B-8B2C-4015-BBAC-438DA5DAB005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -95,9 +95,6 @@
     <t>Make model class for meal</t>
   </si>
   <si>
-    <t>View planner</t>
-  </si>
-  <si>
     <t>Make view for viewing planner</t>
   </si>
   <si>
@@ -126,13 +123,16 @@
   </si>
   <si>
     <t>Estimate Totals</t>
+  </si>
+  <si>
+    <t>View planner (Kirya)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -328,10 +328,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>2.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1423,14 +1423,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G28"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="51.42578125" customWidth="1"/>
     <col min="2" max="2" width="41.7109375" customWidth="1"/>
     <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -1447,7 +1447,7 @@
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="7"/>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
@@ -1464,7 +1464,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -1479,7 +1479,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1494,7 +1494,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -1509,7 +1509,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -1524,7 +1524,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -1539,7 +1539,7 @@
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>12</v>
       </c>
@@ -1554,7 +1554,7 @@
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -1569,7 +1569,7 @@
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -1584,57 +1584,69 @@
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="C11" s="1">
         <v>0.5</v>
       </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
+      <c r="D11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="E11" s="2">
+        <v>0</v>
+      </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C12" s="1">
         <v>1.5</v>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
+      <c r="D12" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="E12" s="2">
+        <v>1.5</v>
+      </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C13" s="1">
         <v>1</v>
       </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+      <c r="D13" s="2">
+        <v>1</v>
+      </c>
+      <c r="E13" s="2">
+        <v>1</v>
+      </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="C14" s="1">
         <v>1.5</v>
@@ -1644,12 +1656,12 @@
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="C15" s="1">
         <v>0.5</v>
@@ -1659,12 +1671,12 @@
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C16" s="1">
         <v>1</v>
@@ -1674,12 +1686,12 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C17" s="1">
         <v>1</v>
@@ -1689,7 +1701,7 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -1698,7 +1710,7 @@
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -1707,7 +1719,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -1716,7 +1728,7 @@
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -1725,7 +1737,7 @@
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -1734,7 +1746,7 @@
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1743,7 +1755,7 @@
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -1752,7 +1764,7 @@
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
     </row>
-    <row r="25" spans="1:7">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -1761,7 +1773,7 @@
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1770,9 +1782,9 @@
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
     </row>
-    <row r="27" spans="1:7">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B27" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C27" s="3">
         <f>SUM(C3:C26)</f>
@@ -1780,11 +1792,11 @@
       </c>
       <c r="D27" s="3">
         <f t="shared" ref="D27:G27" si="0">SUM(D3:D26)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E27" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="F27" s="3">
         <f t="shared" si="0"/>
@@ -1795,7 +1807,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D28">
         <f>$C$27</f>
         <v>14</v>

</xml_diff>